<commit_message>
Update Fate Dioses y monstruos.xlsx
</commit_message>
<xml_diff>
--- a/Fate/Hojas de personaje/Fate Dioses y monstruos.xlsx
+++ b/Fate/Hojas de personaje/Fate Dioses y monstruos.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
   <si>
     <t>Nombre:</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Poderoso:</t>
   </si>
   <si>
-    <t>Grado del Manto</t>
+    <t>Grado Manto</t>
   </si>
   <si>
     <t>Sabio:</t>
@@ -112,7 +112,10 @@
     <t>Estrés y Consecuencias</t>
   </si>
   <si>
-    <t>Estrés</t>
+    <t>Estrés Fisico</t>
+  </si>
+  <si>
+    <t>Estrés Mental</t>
   </si>
   <si>
     <t>Leve</t>
@@ -155,7 +158,7 @@
       <patternFill patternType="lightGray"/>
     </fill>
   </fills>
-  <borders count="63">
+  <borders count="68">
     <border/>
     <border>
       <left style="thick">
@@ -673,6 +676,45 @@
       <left style="thick">
         <color rgb="FF000000"/>
       </left>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF000000"/>
+      </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -684,12 +726,19 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="thick">
         <color rgb="FF000000"/>
       </bottom>
@@ -706,42 +755,9 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
       <right style="thick">
         <color rgb="FF000000"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="thick">
         <color rgb="FF000000"/>
       </bottom>
@@ -750,7 +766,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="95">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -891,33 +907,29 @@
     <xf borderId="44" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="45" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="42" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="46" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="46" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="47" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="48" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="23" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="27" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="27" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="49" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="50" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="50" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="51" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="52" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="53" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -925,26 +937,35 @@
     <xf borderId="55" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="42" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="56" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="12" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="46" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="57" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="56" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="57" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="center"/>
+    <xf borderId="32" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="58" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="59" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="55" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="58" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="59" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="60" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="17" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="61" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="60" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="61" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="50" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="62" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="63" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="64" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="65" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="66" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="67" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1846,39 +1867,39 @@
     </row>
     <row r="23">
       <c r="A23" s="1"/>
-      <c r="B23" s="70" t="s">
+      <c r="B23" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="71"/>
-      <c r="D23" s="72">
+      <c r="C23" s="70"/>
+      <c r="D23" s="32">
         <v>3.0</v>
       </c>
       <c r="E23" s="65"/>
       <c r="F23" s="65"/>
-      <c r="G23" s="72">
+      <c r="G23" s="32">
         <v>2.0</v>
       </c>
       <c r="H23" s="65"/>
-      <c r="I23" s="72">
+      <c r="I23" s="32">
         <v>1.0</v>
       </c>
-      <c r="J23" s="72">
+      <c r="J23" s="32">
         <v>0.0</v>
       </c>
-      <c r="K23" s="72">
+      <c r="K23" s="32">
         <v>1.0</v>
       </c>
       <c r="L23" s="65"/>
-      <c r="M23" s="72">
+      <c r="M23" s="32">
         <v>2.0</v>
       </c>
       <c r="N23" s="65"/>
       <c r="O23" s="65"/>
-      <c r="P23" s="72">
+      <c r="P23" s="32">
         <v>3.0</v>
       </c>
       <c r="Q23" s="65"/>
-      <c r="R23" s="73" t="s">
+      <c r="R23" s="71" t="s">
         <v>29</v>
       </c>
       <c r="S23" s="9"/>
@@ -1922,39 +1943,39 @@
     </row>
     <row r="25">
       <c r="A25" s="1"/>
-      <c r="B25" s="70" t="s">
+      <c r="B25" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="74"/>
-      <c r="D25" s="72">
+      <c r="C25" s="72"/>
+      <c r="D25" s="32">
         <v>3.0</v>
       </c>
       <c r="E25" s="64"/>
       <c r="F25" s="64"/>
-      <c r="G25" s="72">
+      <c r="G25" s="32">
         <v>2.0</v>
       </c>
       <c r="H25" s="65"/>
-      <c r="I25" s="72">
+      <c r="I25" s="32">
         <v>1.0</v>
       </c>
-      <c r="J25" s="72">
+      <c r="J25" s="32">
         <v>0.0</v>
       </c>
-      <c r="K25" s="72">
+      <c r="K25" s="32">
         <v>1.0</v>
       </c>
       <c r="L25" s="65"/>
-      <c r="M25" s="72">
+      <c r="M25" s="32">
         <v>2.0</v>
       </c>
       <c r="N25" s="65"/>
       <c r="O25" s="65"/>
-      <c r="P25" s="72">
+      <c r="P25" s="32">
         <v>3.0</v>
       </c>
       <c r="Q25" s="65"/>
-      <c r="R25" s="73" t="s">
+      <c r="R25" s="71" t="s">
         <v>31</v>
       </c>
       <c r="S25" s="9"/>
@@ -1969,23 +1990,23 @@
     </row>
     <row r="26">
       <c r="A26" s="1"/>
-      <c r="B26" s="75"/>
-      <c r="C26" s="76"/>
-      <c r="D26" s="77"/>
-      <c r="E26" s="77"/>
-      <c r="F26" s="77"/>
-      <c r="G26" s="77"/>
-      <c r="H26" s="77"/>
-      <c r="I26" s="77"/>
-      <c r="J26" s="77"/>
-      <c r="K26" s="77"/>
-      <c r="L26" s="77"/>
-      <c r="M26" s="77"/>
-      <c r="N26" s="77"/>
-      <c r="O26" s="77"/>
-      <c r="P26" s="77"/>
-      <c r="Q26" s="77"/>
-      <c r="R26" s="78"/>
+      <c r="B26" s="73"/>
+      <c r="C26" s="74"/>
+      <c r="D26" s="75"/>
+      <c r="E26" s="75"/>
+      <c r="F26" s="75"/>
+      <c r="G26" s="75"/>
+      <c r="H26" s="75"/>
+      <c r="I26" s="75"/>
+      <c r="J26" s="75"/>
+      <c r="K26" s="75"/>
+      <c r="L26" s="75"/>
+      <c r="M26" s="75"/>
+      <c r="N26" s="75"/>
+      <c r="O26" s="75"/>
+      <c r="P26" s="75"/>
+      <c r="Q26" s="75"/>
+      <c r="R26" s="76"/>
       <c r="S26" s="1"/>
       <c r="T26" s="1"/>
       <c r="U26" s="1"/>
@@ -1999,7 +2020,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1"/>
-      <c r="B27" s="79" t="s">
+      <c r="B27" s="77" t="s">
         <v>32</v>
       </c>
       <c r="C27" s="21"/>
@@ -2031,39 +2052,43 @@
     </row>
     <row r="28">
       <c r="A28" s="1"/>
-      <c r="B28" s="80" t="s">
+      <c r="B28" s="78" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="19">
+      <c r="C28" s="16">
         <v>1.0</v>
       </c>
-      <c r="D28" s="19">
+      <c r="D28" s="18"/>
+      <c r="E28" s="16">
         <v>2.0</v>
       </c>
-      <c r="E28" s="19">
+      <c r="F28" s="18"/>
+      <c r="G28" s="16">
         <v>3.0</v>
       </c>
-      <c r="F28" s="81">
+      <c r="H28" s="18"/>
+      <c r="I28" s="79">
         <v>4.0</v>
       </c>
-      <c r="G28" s="82" t="s">
+      <c r="J28" s="41"/>
+      <c r="K28" s="80" t="s">
         <v>34</v>
       </c>
-      <c r="H28" s="38"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="82" t="s">
-        <v>35</v>
+      <c r="L28" s="16">
+        <v>1.0</v>
       </c>
-      <c r="L28" s="38"/>
-      <c r="M28" s="17"/>
-      <c r="N28" s="18"/>
-      <c r="O28" s="82" t="s">
-        <v>36</v>
+      <c r="M28" s="18"/>
+      <c r="N28" s="16">
+        <v>2.0</v>
       </c>
-      <c r="P28" s="38"/>
-      <c r="Q28" s="17"/>
-      <c r="R28" s="39"/>
+      <c r="O28" s="18"/>
+      <c r="P28" s="16">
+        <v>3.0</v>
+      </c>
+      <c r="Q28" s="18"/>
+      <c r="R28" s="81">
+        <v>4.0</v>
+      </c>
       <c r="S28" s="1"/>
       <c r="T28" s="1"/>
       <c r="U28" s="1"/>
@@ -2077,23 +2102,23 @@
     </row>
     <row r="29">
       <c r="A29" s="1"/>
-      <c r="B29" s="83"/>
-      <c r="C29" s="84"/>
-      <c r="D29" s="84"/>
-      <c r="E29" s="84"/>
-      <c r="F29" s="84"/>
-      <c r="G29" s="85"/>
-      <c r="H29" s="86"/>
-      <c r="I29" s="87"/>
-      <c r="J29" s="88"/>
+      <c r="B29" s="82"/>
+      <c r="C29" s="83"/>
+      <c r="D29" s="74"/>
+      <c r="E29" s="83"/>
+      <c r="F29" s="74"/>
+      <c r="G29" s="83"/>
+      <c r="H29" s="74"/>
+      <c r="I29" s="83"/>
+      <c r="J29" s="84"/>
       <c r="K29" s="85"/>
-      <c r="L29" s="86"/>
-      <c r="M29" s="87"/>
-      <c r="N29" s="88"/>
-      <c r="O29" s="85"/>
-      <c r="P29" s="86"/>
-      <c r="Q29" s="87"/>
-      <c r="R29" s="89"/>
+      <c r="L29" s="83"/>
+      <c r="M29" s="74"/>
+      <c r="N29" s="83"/>
+      <c r="O29" s="74"/>
+      <c r="P29" s="83"/>
+      <c r="Q29" s="74"/>
+      <c r="R29" s="86"/>
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
       <c r="U29" s="1"/>
@@ -2107,11 +2132,21 @@
     </row>
     <row r="30">
       <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
+      <c r="B30" s="63" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="87"/>
+      <c r="G30" s="88"/>
+      <c r="H30" s="65" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" s="87"/>
+      <c r="M30" s="88"/>
+      <c r="N30" s="65" t="s">
+        <v>37</v>
+      </c>
+      <c r="O30" s="87"/>
+      <c r="R30" s="13"/>
       <c r="S30" s="1"/>
       <c r="T30" s="1"/>
       <c r="U30" s="1"/>
@@ -2125,11 +2160,23 @@
     </row>
     <row r="31">
       <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
+      <c r="B31" s="89"/>
+      <c r="C31" s="90"/>
+      <c r="D31" s="91"/>
+      <c r="E31" s="91"/>
+      <c r="F31" s="91"/>
+      <c r="G31" s="92"/>
+      <c r="H31" s="93"/>
+      <c r="I31" s="90"/>
+      <c r="J31" s="91"/>
+      <c r="K31" s="91"/>
+      <c r="L31" s="91"/>
+      <c r="M31" s="92"/>
+      <c r="N31" s="93"/>
+      <c r="O31" s="90"/>
+      <c r="P31" s="91"/>
+      <c r="Q31" s="91"/>
+      <c r="R31" s="94"/>
       <c r="S31" s="1"/>
       <c r="T31" s="1"/>
       <c r="U31" s="1"/>
@@ -31212,7 +31259,7 @@
       <c r="AB1000" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="106">
+  <mergeCells count="118">
     <mergeCell ref="K6:R6"/>
     <mergeCell ref="J7:R7"/>
     <mergeCell ref="K8:R8"/>
@@ -31245,6 +31292,58 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="C17:I17"/>
     <mergeCell ref="C18:I18"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="K14:R14"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="K15:R15"/>
+    <mergeCell ref="C16:I16"/>
+    <mergeCell ref="J16:R16"/>
+    <mergeCell ref="J17:R19"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="K21:K22"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="M21:M22"/>
+    <mergeCell ref="N21:N22"/>
+    <mergeCell ref="O21:O22"/>
+    <mergeCell ref="P21:P22"/>
+    <mergeCell ref="Q21:Q22"/>
+    <mergeCell ref="R21:R22"/>
+    <mergeCell ref="W21:Y21"/>
+    <mergeCell ref="W22:Y22"/>
+    <mergeCell ref="W23:Y23"/>
+    <mergeCell ref="C19:I19"/>
+    <mergeCell ref="B20:R20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="P28:Q28"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="H30:H31"/>
+    <mergeCell ref="N30:N31"/>
+    <mergeCell ref="O30:R31"/>
+    <mergeCell ref="K28:K29"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I30:M31"/>
+    <mergeCell ref="C30:G31"/>
+    <mergeCell ref="L28:M28"/>
     <mergeCell ref="N23:N24"/>
     <mergeCell ref="O23:O24"/>
     <mergeCell ref="P23:P24"/>
@@ -31275,50 +31374,10 @@
     <mergeCell ref="N25:N26"/>
     <mergeCell ref="O25:O26"/>
     <mergeCell ref="B27:R27"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="K28:K29"/>
-    <mergeCell ref="L28:N28"/>
-    <mergeCell ref="O28:O29"/>
-    <mergeCell ref="P28:R28"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="P29:R29"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="H25:H26"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="K14:R14"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="K15:R15"/>
-    <mergeCell ref="C16:I16"/>
-    <mergeCell ref="J16:R16"/>
-    <mergeCell ref="J17:R19"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="K21:K22"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="M21:M22"/>
-    <mergeCell ref="N21:N22"/>
-    <mergeCell ref="O21:O22"/>
-    <mergeCell ref="P21:P22"/>
-    <mergeCell ref="Q21:Q22"/>
-    <mergeCell ref="R21:R22"/>
-    <mergeCell ref="W21:Y21"/>
-    <mergeCell ref="W22:Y22"/>
-    <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="C19:I19"/>
-    <mergeCell ref="B20:R20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="P29:Q29"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>